<commit_message>
Updated BAADTbVT and AVLo data using E+ database
</commit_message>
<xml_diff>
--- a/InputData/trans/AVLo/Avg Vehicle Loading.xlsx
+++ b/InputData/trans/AVLo/Avg Vehicle Loading.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28324"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anima\OneDrive\Desktop\Models\eps-brazil-cpl2\InputData\trans\AVLo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saido\Documents\eps-brazil-cpl\InputData\trans\AVLo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BE2088D-E54A-4460-8D4F-1648AA57E0A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="21795" windowHeight="12975" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -29,7 +28,7 @@
     <definedName name="ti_tbl_50">#REF!</definedName>
     <definedName name="ti_tbl_69">#REF!</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -398,7 +397,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="6">
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
@@ -1298,160 +1297,160 @@
     </xf>
   </cellXfs>
   <cellStyles count="154">
-    <cellStyle name="20% - Accent1 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
-    <cellStyle name="20% - Accent2 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
-    <cellStyle name="20% - Accent3 2" xfId="4" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
-    <cellStyle name="20% - Accent4 2" xfId="5" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
-    <cellStyle name="20% - Accent5 2" xfId="6" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
-    <cellStyle name="20% - Accent6 2" xfId="7" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
-    <cellStyle name="40% - Accent1 2" xfId="8" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
-    <cellStyle name="40% - Accent2 2" xfId="9" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
-    <cellStyle name="40% - Accent3 2" xfId="10" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
-    <cellStyle name="40% - Accent4 2" xfId="11" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
-    <cellStyle name="40% - Accent5 2" xfId="12" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
-    <cellStyle name="40% - Accent6 2" xfId="13" xr:uid="{00000000-0005-0000-0000-00000B000000}"/>
-    <cellStyle name="60% - Accent1 2" xfId="14" xr:uid="{00000000-0005-0000-0000-00000C000000}"/>
-    <cellStyle name="60% - Accent2 2" xfId="15" xr:uid="{00000000-0005-0000-0000-00000D000000}"/>
-    <cellStyle name="60% - Accent3 2" xfId="16" xr:uid="{00000000-0005-0000-0000-00000E000000}"/>
-    <cellStyle name="60% - Accent4 2" xfId="17" xr:uid="{00000000-0005-0000-0000-00000F000000}"/>
-    <cellStyle name="60% - Accent5 2" xfId="18" xr:uid="{00000000-0005-0000-0000-000010000000}"/>
-    <cellStyle name="60% - Accent6 2" xfId="19" xr:uid="{00000000-0005-0000-0000-000011000000}"/>
-    <cellStyle name="Accent1 2" xfId="20" xr:uid="{00000000-0005-0000-0000-000012000000}"/>
-    <cellStyle name="Accent2 2" xfId="21" xr:uid="{00000000-0005-0000-0000-000013000000}"/>
-    <cellStyle name="Accent3 2" xfId="22" xr:uid="{00000000-0005-0000-0000-000014000000}"/>
-    <cellStyle name="Accent4 2" xfId="23" xr:uid="{00000000-0005-0000-0000-000015000000}"/>
-    <cellStyle name="Accent5 2" xfId="24" xr:uid="{00000000-0005-0000-0000-000016000000}"/>
-    <cellStyle name="Accent6 2" xfId="25" xr:uid="{00000000-0005-0000-0000-000017000000}"/>
-    <cellStyle name="Bad 2" xfId="26" xr:uid="{00000000-0005-0000-0000-000018000000}"/>
-    <cellStyle name="Body: normal cell" xfId="27" xr:uid="{00000000-0005-0000-0000-000019000000}"/>
-    <cellStyle name="Body: normal cell 2" xfId="28" xr:uid="{00000000-0005-0000-0000-00001A000000}"/>
-    <cellStyle name="Calculation 2" xfId="29" xr:uid="{00000000-0005-0000-0000-00001B000000}"/>
-    <cellStyle name="Check Cell 2" xfId="30" xr:uid="{00000000-0005-0000-0000-00001C000000}"/>
-    <cellStyle name="Column heading" xfId="31" xr:uid="{00000000-0005-0000-0000-00001D000000}"/>
-    <cellStyle name="Comma 2" xfId="32" xr:uid="{00000000-0005-0000-0000-00001E000000}"/>
-    <cellStyle name="Comma 2 2" xfId="33" xr:uid="{00000000-0005-0000-0000-00001F000000}"/>
-    <cellStyle name="Comma 3" xfId="34" xr:uid="{00000000-0005-0000-0000-000020000000}"/>
-    <cellStyle name="Comma 4" xfId="35" xr:uid="{00000000-0005-0000-0000-000021000000}"/>
-    <cellStyle name="Comma 5" xfId="36" xr:uid="{00000000-0005-0000-0000-000022000000}"/>
-    <cellStyle name="Comma 6" xfId="37" xr:uid="{00000000-0005-0000-0000-000023000000}"/>
-    <cellStyle name="Comma 7" xfId="38" xr:uid="{00000000-0005-0000-0000-000024000000}"/>
-    <cellStyle name="Comma 8" xfId="39" xr:uid="{00000000-0005-0000-0000-000025000000}"/>
-    <cellStyle name="Corner heading" xfId="40" xr:uid="{00000000-0005-0000-0000-000026000000}"/>
-    <cellStyle name="Currency 2" xfId="41" xr:uid="{00000000-0005-0000-0000-000027000000}"/>
-    <cellStyle name="Currency 3" xfId="42" xr:uid="{00000000-0005-0000-0000-000028000000}"/>
-    <cellStyle name="Currency 3 2" xfId="43" xr:uid="{00000000-0005-0000-0000-000029000000}"/>
-    <cellStyle name="Data" xfId="44" xr:uid="{00000000-0005-0000-0000-00002A000000}"/>
-    <cellStyle name="Data 2" xfId="45" xr:uid="{00000000-0005-0000-0000-00002B000000}"/>
-    <cellStyle name="Data no deci" xfId="46" xr:uid="{00000000-0005-0000-0000-00002C000000}"/>
-    <cellStyle name="Data Superscript" xfId="47" xr:uid="{00000000-0005-0000-0000-00002D000000}"/>
-    <cellStyle name="Data_1-1A-Regular" xfId="48" xr:uid="{00000000-0005-0000-0000-00002E000000}"/>
-    <cellStyle name="Explanatory Text 2" xfId="49" xr:uid="{00000000-0005-0000-0000-00002F000000}"/>
-    <cellStyle name="Font: Calibri, 9pt regular" xfId="50" xr:uid="{00000000-0005-0000-0000-000030000000}"/>
-    <cellStyle name="Font: Calibri, 9pt regular 2" xfId="51" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
-    <cellStyle name="Footnotes: top row" xfId="52" xr:uid="{00000000-0005-0000-0000-000032000000}"/>
-    <cellStyle name="Footnotes: top row 2" xfId="53" xr:uid="{00000000-0005-0000-0000-000033000000}"/>
-    <cellStyle name="Good 2" xfId="54" xr:uid="{00000000-0005-0000-0000-000034000000}"/>
-    <cellStyle name="Header: bottom row" xfId="55" xr:uid="{00000000-0005-0000-0000-000035000000}"/>
-    <cellStyle name="Header: bottom row 2" xfId="56" xr:uid="{00000000-0005-0000-0000-000036000000}"/>
-    <cellStyle name="Heading 1 2" xfId="57" xr:uid="{00000000-0005-0000-0000-000037000000}"/>
-    <cellStyle name="Heading 2 2" xfId="58" xr:uid="{00000000-0005-0000-0000-000038000000}"/>
-    <cellStyle name="Heading 3 2" xfId="59" xr:uid="{00000000-0005-0000-0000-000039000000}"/>
-    <cellStyle name="Heading 4 2" xfId="60" xr:uid="{00000000-0005-0000-0000-00003A000000}"/>
-    <cellStyle name="Hed Side" xfId="61" xr:uid="{00000000-0005-0000-0000-00003B000000}"/>
-    <cellStyle name="Hed Side 2" xfId="62" xr:uid="{00000000-0005-0000-0000-00003C000000}"/>
-    <cellStyle name="Hed Side bold" xfId="63" xr:uid="{00000000-0005-0000-0000-00003D000000}"/>
-    <cellStyle name="Hed Side Indent" xfId="64" xr:uid="{00000000-0005-0000-0000-00003E000000}"/>
-    <cellStyle name="Hed Side Regular" xfId="65" xr:uid="{00000000-0005-0000-0000-00003F000000}"/>
-    <cellStyle name="Hed Side_1-1A-Regular" xfId="66" xr:uid="{00000000-0005-0000-0000-000040000000}"/>
-    <cellStyle name="Hed Top" xfId="67" xr:uid="{00000000-0005-0000-0000-000041000000}"/>
-    <cellStyle name="Hed Top - SECTION" xfId="68" xr:uid="{00000000-0005-0000-0000-000042000000}"/>
-    <cellStyle name="Hed Top_3-new4" xfId="69" xr:uid="{00000000-0005-0000-0000-000043000000}"/>
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
-    <cellStyle name="Hyperlink 2" xfId="70" xr:uid="{00000000-0005-0000-0000-000045000000}"/>
-    <cellStyle name="Input 2" xfId="71" xr:uid="{00000000-0005-0000-0000-000046000000}"/>
-    <cellStyle name="Linked Cell 2" xfId="72" xr:uid="{00000000-0005-0000-0000-000047000000}"/>
-    <cellStyle name="Neutral 2" xfId="73" xr:uid="{00000000-0005-0000-0000-000048000000}"/>
+    <cellStyle name="20% - Accent1 2" xfId="2"/>
+    <cellStyle name="20% - Accent2 2" xfId="3"/>
+    <cellStyle name="20% - Accent3 2" xfId="4"/>
+    <cellStyle name="20% - Accent4 2" xfId="5"/>
+    <cellStyle name="20% - Accent5 2" xfId="6"/>
+    <cellStyle name="20% - Accent6 2" xfId="7"/>
+    <cellStyle name="40% - Accent1 2" xfId="8"/>
+    <cellStyle name="40% - Accent2 2" xfId="9"/>
+    <cellStyle name="40% - Accent3 2" xfId="10"/>
+    <cellStyle name="40% - Accent4 2" xfId="11"/>
+    <cellStyle name="40% - Accent5 2" xfId="12"/>
+    <cellStyle name="40% - Accent6 2" xfId="13"/>
+    <cellStyle name="60% - Accent1 2" xfId="14"/>
+    <cellStyle name="60% - Accent2 2" xfId="15"/>
+    <cellStyle name="60% - Accent3 2" xfId="16"/>
+    <cellStyle name="60% - Accent4 2" xfId="17"/>
+    <cellStyle name="60% - Accent5 2" xfId="18"/>
+    <cellStyle name="60% - Accent6 2" xfId="19"/>
+    <cellStyle name="Accent1 2" xfId="20"/>
+    <cellStyle name="Accent2 2" xfId="21"/>
+    <cellStyle name="Accent3 2" xfId="22"/>
+    <cellStyle name="Accent4 2" xfId="23"/>
+    <cellStyle name="Accent5 2" xfId="24"/>
+    <cellStyle name="Accent6 2" xfId="25"/>
+    <cellStyle name="Bad 2" xfId="26"/>
+    <cellStyle name="Body: normal cell" xfId="27"/>
+    <cellStyle name="Body: normal cell 2" xfId="28"/>
+    <cellStyle name="Calculation 2" xfId="29"/>
+    <cellStyle name="Check Cell 2" xfId="30"/>
+    <cellStyle name="Column heading" xfId="31"/>
+    <cellStyle name="Comma 2" xfId="32"/>
+    <cellStyle name="Comma 2 2" xfId="33"/>
+    <cellStyle name="Comma 3" xfId="34"/>
+    <cellStyle name="Comma 4" xfId="35"/>
+    <cellStyle name="Comma 5" xfId="36"/>
+    <cellStyle name="Comma 6" xfId="37"/>
+    <cellStyle name="Comma 7" xfId="38"/>
+    <cellStyle name="Comma 8" xfId="39"/>
+    <cellStyle name="Corner heading" xfId="40"/>
+    <cellStyle name="Currency 2" xfId="41"/>
+    <cellStyle name="Currency 3" xfId="42"/>
+    <cellStyle name="Currency 3 2" xfId="43"/>
+    <cellStyle name="Data" xfId="44"/>
+    <cellStyle name="Data 2" xfId="45"/>
+    <cellStyle name="Data no deci" xfId="46"/>
+    <cellStyle name="Data Superscript" xfId="47"/>
+    <cellStyle name="Data_1-1A-Regular" xfId="48"/>
+    <cellStyle name="Explanatory Text 2" xfId="49"/>
+    <cellStyle name="Font: Calibri, 9pt regular" xfId="50"/>
+    <cellStyle name="Font: Calibri, 9pt regular 2" xfId="51"/>
+    <cellStyle name="Footnotes: top row" xfId="52"/>
+    <cellStyle name="Footnotes: top row 2" xfId="53"/>
+    <cellStyle name="Good 2" xfId="54"/>
+    <cellStyle name="Header: bottom row" xfId="55"/>
+    <cellStyle name="Header: bottom row 2" xfId="56"/>
+    <cellStyle name="Heading 1 2" xfId="57"/>
+    <cellStyle name="Heading 2 2" xfId="58"/>
+    <cellStyle name="Heading 3 2" xfId="59"/>
+    <cellStyle name="Heading 4 2" xfId="60"/>
+    <cellStyle name="Hed Side" xfId="61"/>
+    <cellStyle name="Hed Side 2" xfId="62"/>
+    <cellStyle name="Hed Side bold" xfId="63"/>
+    <cellStyle name="Hed Side Indent" xfId="64"/>
+    <cellStyle name="Hed Side Regular" xfId="65"/>
+    <cellStyle name="Hed Side_1-1A-Regular" xfId="66"/>
+    <cellStyle name="Hed Top" xfId="67"/>
+    <cellStyle name="Hed Top - SECTION" xfId="68"/>
+    <cellStyle name="Hed Top_3-new4" xfId="69"/>
+    <cellStyle name="Hyperlink 2" xfId="70"/>
+    <cellStyle name="Input 2" xfId="71"/>
+    <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
+    <cellStyle name="Linked Cell 2" xfId="72"/>
+    <cellStyle name="Neutral 2" xfId="73"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 10" xfId="74" xr:uid="{00000000-0005-0000-0000-00004A000000}"/>
-    <cellStyle name="Normal 11" xfId="75" xr:uid="{00000000-0005-0000-0000-00004B000000}"/>
-    <cellStyle name="Normal 2" xfId="76" xr:uid="{00000000-0005-0000-0000-00004C000000}"/>
-    <cellStyle name="Normal 2 2" xfId="77" xr:uid="{00000000-0005-0000-0000-00004D000000}"/>
-    <cellStyle name="Normal 2 3" xfId="78" xr:uid="{00000000-0005-0000-0000-00004E000000}"/>
-    <cellStyle name="Normal 3" xfId="79" xr:uid="{00000000-0005-0000-0000-00004F000000}"/>
-    <cellStyle name="Normal 3 2" xfId="80" xr:uid="{00000000-0005-0000-0000-000050000000}"/>
-    <cellStyle name="Normal 3 2 2" xfId="81" xr:uid="{00000000-0005-0000-0000-000051000000}"/>
-    <cellStyle name="Normal 3 2 2 2" xfId="82" xr:uid="{00000000-0005-0000-0000-000052000000}"/>
-    <cellStyle name="Normal 3 2 3" xfId="83" xr:uid="{00000000-0005-0000-0000-000053000000}"/>
-    <cellStyle name="Normal 3 3" xfId="84" xr:uid="{00000000-0005-0000-0000-000054000000}"/>
-    <cellStyle name="Normal 3 3 2" xfId="85" xr:uid="{00000000-0005-0000-0000-000055000000}"/>
-    <cellStyle name="Normal 3 3 2 2" xfId="86" xr:uid="{00000000-0005-0000-0000-000056000000}"/>
-    <cellStyle name="Normal 3 3 3" xfId="87" xr:uid="{00000000-0005-0000-0000-000057000000}"/>
-    <cellStyle name="Normal 3 4" xfId="88" xr:uid="{00000000-0005-0000-0000-000058000000}"/>
-    <cellStyle name="Normal 3 4 2" xfId="89" xr:uid="{00000000-0005-0000-0000-000059000000}"/>
-    <cellStyle name="Normal 3 5" xfId="90" xr:uid="{00000000-0005-0000-0000-00005A000000}"/>
-    <cellStyle name="Normal 3 6" xfId="91" xr:uid="{00000000-0005-0000-0000-00005B000000}"/>
-    <cellStyle name="Normal 3 7" xfId="92" xr:uid="{00000000-0005-0000-0000-00005C000000}"/>
-    <cellStyle name="Normal 4" xfId="93" xr:uid="{00000000-0005-0000-0000-00005D000000}"/>
-    <cellStyle name="Normal 4 2" xfId="94" xr:uid="{00000000-0005-0000-0000-00005E000000}"/>
-    <cellStyle name="Normal 4 2 2" xfId="95" xr:uid="{00000000-0005-0000-0000-00005F000000}"/>
-    <cellStyle name="Normal 4 2 2 2" xfId="96" xr:uid="{00000000-0005-0000-0000-000060000000}"/>
-    <cellStyle name="Normal 4 2 3" xfId="97" xr:uid="{00000000-0005-0000-0000-000061000000}"/>
-    <cellStyle name="Normal 4 3" xfId="98" xr:uid="{00000000-0005-0000-0000-000062000000}"/>
-    <cellStyle name="Normal 4 3 2" xfId="99" xr:uid="{00000000-0005-0000-0000-000063000000}"/>
-    <cellStyle name="Normal 4 3 2 2" xfId="100" xr:uid="{00000000-0005-0000-0000-000064000000}"/>
-    <cellStyle name="Normal 4 3 3" xfId="101" xr:uid="{00000000-0005-0000-0000-000065000000}"/>
-    <cellStyle name="Normal 4 4" xfId="102" xr:uid="{00000000-0005-0000-0000-000066000000}"/>
-    <cellStyle name="Normal 4 4 2" xfId="103" xr:uid="{00000000-0005-0000-0000-000067000000}"/>
-    <cellStyle name="Normal 4 5" xfId="104" xr:uid="{00000000-0005-0000-0000-000068000000}"/>
-    <cellStyle name="Normal 4 6" xfId="105" xr:uid="{00000000-0005-0000-0000-000069000000}"/>
-    <cellStyle name="Normal 4 7" xfId="106" xr:uid="{00000000-0005-0000-0000-00006A000000}"/>
-    <cellStyle name="Normal 5" xfId="107" xr:uid="{00000000-0005-0000-0000-00006B000000}"/>
-    <cellStyle name="Normal 5 2" xfId="108" xr:uid="{00000000-0005-0000-0000-00006C000000}"/>
-    <cellStyle name="Normal 5 3" xfId="109" xr:uid="{00000000-0005-0000-0000-00006D000000}"/>
-    <cellStyle name="Normal 6" xfId="110" xr:uid="{00000000-0005-0000-0000-00006E000000}"/>
-    <cellStyle name="Normal 6 2" xfId="111" xr:uid="{00000000-0005-0000-0000-00006F000000}"/>
-    <cellStyle name="Normal 7" xfId="112" xr:uid="{00000000-0005-0000-0000-000070000000}"/>
-    <cellStyle name="Normal 7 2" xfId="113" xr:uid="{00000000-0005-0000-0000-000071000000}"/>
-    <cellStyle name="Normal 8" xfId="114" xr:uid="{00000000-0005-0000-0000-000072000000}"/>
-    <cellStyle name="Normal 9" xfId="115" xr:uid="{00000000-0005-0000-0000-000073000000}"/>
-    <cellStyle name="Note 2" xfId="116" xr:uid="{00000000-0005-0000-0000-000074000000}"/>
-    <cellStyle name="Note 2 2" xfId="117" xr:uid="{00000000-0005-0000-0000-000075000000}"/>
-    <cellStyle name="Output 2" xfId="118" xr:uid="{00000000-0005-0000-0000-000076000000}"/>
-    <cellStyle name="Parent row" xfId="119" xr:uid="{00000000-0005-0000-0000-000077000000}"/>
-    <cellStyle name="Parent row 2" xfId="120" xr:uid="{00000000-0005-0000-0000-000078000000}"/>
-    <cellStyle name="Percent 2" xfId="121" xr:uid="{00000000-0005-0000-0000-000079000000}"/>
-    <cellStyle name="Percent 2 2" xfId="122" xr:uid="{00000000-0005-0000-0000-00007A000000}"/>
-    <cellStyle name="Percent 3" xfId="123" xr:uid="{00000000-0005-0000-0000-00007B000000}"/>
-    <cellStyle name="Percent 3 2" xfId="124" xr:uid="{00000000-0005-0000-0000-00007C000000}"/>
-    <cellStyle name="Percent 4" xfId="125" xr:uid="{00000000-0005-0000-0000-00007D000000}"/>
-    <cellStyle name="Reference" xfId="126" xr:uid="{00000000-0005-0000-0000-00007E000000}"/>
-    <cellStyle name="Row heading" xfId="127" xr:uid="{00000000-0005-0000-0000-00007F000000}"/>
-    <cellStyle name="Source Hed" xfId="128" xr:uid="{00000000-0005-0000-0000-000080000000}"/>
-    <cellStyle name="Source Letter" xfId="129" xr:uid="{00000000-0005-0000-0000-000081000000}"/>
-    <cellStyle name="Source Superscript" xfId="130" xr:uid="{00000000-0005-0000-0000-000082000000}"/>
-    <cellStyle name="Source Superscript 2" xfId="131" xr:uid="{00000000-0005-0000-0000-000083000000}"/>
-    <cellStyle name="Source Text" xfId="132" xr:uid="{00000000-0005-0000-0000-000084000000}"/>
-    <cellStyle name="Source Text 2" xfId="133" xr:uid="{00000000-0005-0000-0000-000085000000}"/>
-    <cellStyle name="State" xfId="134" xr:uid="{00000000-0005-0000-0000-000086000000}"/>
-    <cellStyle name="Superscript" xfId="135" xr:uid="{00000000-0005-0000-0000-000087000000}"/>
-    <cellStyle name="Table Data" xfId="136" xr:uid="{00000000-0005-0000-0000-000088000000}"/>
-    <cellStyle name="Table Head Top" xfId="137" xr:uid="{00000000-0005-0000-0000-000089000000}"/>
-    <cellStyle name="Table Hed Side" xfId="138" xr:uid="{00000000-0005-0000-0000-00008A000000}"/>
-    <cellStyle name="Table title" xfId="139" xr:uid="{00000000-0005-0000-0000-00008B000000}"/>
-    <cellStyle name="Table title 2" xfId="140" xr:uid="{00000000-0005-0000-0000-00008C000000}"/>
-    <cellStyle name="Title 2" xfId="141" xr:uid="{00000000-0005-0000-0000-00008D000000}"/>
-    <cellStyle name="Title Text" xfId="142" xr:uid="{00000000-0005-0000-0000-00008E000000}"/>
-    <cellStyle name="Title Text 1" xfId="143" xr:uid="{00000000-0005-0000-0000-00008F000000}"/>
-    <cellStyle name="Title Text 2" xfId="144" xr:uid="{00000000-0005-0000-0000-000090000000}"/>
-    <cellStyle name="Title-1" xfId="145" xr:uid="{00000000-0005-0000-0000-000091000000}"/>
-    <cellStyle name="Title-2" xfId="146" xr:uid="{00000000-0005-0000-0000-000092000000}"/>
-    <cellStyle name="Title-3" xfId="147" xr:uid="{00000000-0005-0000-0000-000093000000}"/>
-    <cellStyle name="Total 2" xfId="148" xr:uid="{00000000-0005-0000-0000-000094000000}"/>
-    <cellStyle name="Warning Text 2" xfId="149" xr:uid="{00000000-0005-0000-0000-000095000000}"/>
-    <cellStyle name="Wrap" xfId="150" xr:uid="{00000000-0005-0000-0000-000096000000}"/>
-    <cellStyle name="Wrap Bold" xfId="151" xr:uid="{00000000-0005-0000-0000-000097000000}"/>
-    <cellStyle name="Wrap Title" xfId="152" xr:uid="{00000000-0005-0000-0000-000098000000}"/>
-    <cellStyle name="Wrap_NTS99-~11" xfId="153" xr:uid="{00000000-0005-0000-0000-000099000000}"/>
+    <cellStyle name="Normal 10" xfId="74"/>
+    <cellStyle name="Normal 11" xfId="75"/>
+    <cellStyle name="Normal 2" xfId="76"/>
+    <cellStyle name="Normal 2 2" xfId="77"/>
+    <cellStyle name="Normal 2 3" xfId="78"/>
+    <cellStyle name="Normal 3" xfId="79"/>
+    <cellStyle name="Normal 3 2" xfId="80"/>
+    <cellStyle name="Normal 3 2 2" xfId="81"/>
+    <cellStyle name="Normal 3 2 2 2" xfId="82"/>
+    <cellStyle name="Normal 3 2 3" xfId="83"/>
+    <cellStyle name="Normal 3 3" xfId="84"/>
+    <cellStyle name="Normal 3 3 2" xfId="85"/>
+    <cellStyle name="Normal 3 3 2 2" xfId="86"/>
+    <cellStyle name="Normal 3 3 3" xfId="87"/>
+    <cellStyle name="Normal 3 4" xfId="88"/>
+    <cellStyle name="Normal 3 4 2" xfId="89"/>
+    <cellStyle name="Normal 3 5" xfId="90"/>
+    <cellStyle name="Normal 3 6" xfId="91"/>
+    <cellStyle name="Normal 3 7" xfId="92"/>
+    <cellStyle name="Normal 4" xfId="93"/>
+    <cellStyle name="Normal 4 2" xfId="94"/>
+    <cellStyle name="Normal 4 2 2" xfId="95"/>
+    <cellStyle name="Normal 4 2 2 2" xfId="96"/>
+    <cellStyle name="Normal 4 2 3" xfId="97"/>
+    <cellStyle name="Normal 4 3" xfId="98"/>
+    <cellStyle name="Normal 4 3 2" xfId="99"/>
+    <cellStyle name="Normal 4 3 2 2" xfId="100"/>
+    <cellStyle name="Normal 4 3 3" xfId="101"/>
+    <cellStyle name="Normal 4 4" xfId="102"/>
+    <cellStyle name="Normal 4 4 2" xfId="103"/>
+    <cellStyle name="Normal 4 5" xfId="104"/>
+    <cellStyle name="Normal 4 6" xfId="105"/>
+    <cellStyle name="Normal 4 7" xfId="106"/>
+    <cellStyle name="Normal 5" xfId="107"/>
+    <cellStyle name="Normal 5 2" xfId="108"/>
+    <cellStyle name="Normal 5 3" xfId="109"/>
+    <cellStyle name="Normal 6" xfId="110"/>
+    <cellStyle name="Normal 6 2" xfId="111"/>
+    <cellStyle name="Normal 7" xfId="112"/>
+    <cellStyle name="Normal 7 2" xfId="113"/>
+    <cellStyle name="Normal 8" xfId="114"/>
+    <cellStyle name="Normal 9" xfId="115"/>
+    <cellStyle name="Note 2" xfId="116"/>
+    <cellStyle name="Note 2 2" xfId="117"/>
+    <cellStyle name="Output 2" xfId="118"/>
+    <cellStyle name="Parent row" xfId="119"/>
+    <cellStyle name="Parent row 2" xfId="120"/>
+    <cellStyle name="Percent 2" xfId="121"/>
+    <cellStyle name="Percent 2 2" xfId="122"/>
+    <cellStyle name="Percent 3" xfId="123"/>
+    <cellStyle name="Percent 3 2" xfId="124"/>
+    <cellStyle name="Percent 4" xfId="125"/>
+    <cellStyle name="Reference" xfId="126"/>
+    <cellStyle name="Row heading" xfId="127"/>
+    <cellStyle name="Source Hed" xfId="128"/>
+    <cellStyle name="Source Letter" xfId="129"/>
+    <cellStyle name="Source Superscript" xfId="130"/>
+    <cellStyle name="Source Superscript 2" xfId="131"/>
+    <cellStyle name="Source Text" xfId="132"/>
+    <cellStyle name="Source Text 2" xfId="133"/>
+    <cellStyle name="State" xfId="134"/>
+    <cellStyle name="Superscript" xfId="135"/>
+    <cellStyle name="Table Data" xfId="136"/>
+    <cellStyle name="Table Head Top" xfId="137"/>
+    <cellStyle name="Table Hed Side" xfId="138"/>
+    <cellStyle name="Table title" xfId="139"/>
+    <cellStyle name="Table title 2" xfId="140"/>
+    <cellStyle name="Title 2" xfId="141"/>
+    <cellStyle name="Title Text" xfId="142"/>
+    <cellStyle name="Title Text 1" xfId="143"/>
+    <cellStyle name="Title Text 2" xfId="144"/>
+    <cellStyle name="Title-1" xfId="145"/>
+    <cellStyle name="Title-2" xfId="146"/>
+    <cellStyle name="Title-3" xfId="147"/>
+    <cellStyle name="Total 2" xfId="148"/>
+    <cellStyle name="Warning Text 2" xfId="149"/>
+    <cellStyle name="Wrap" xfId="150"/>
+    <cellStyle name="Wrap Bold" xfId="151"/>
+    <cellStyle name="Wrap Title" xfId="152"/>
+    <cellStyle name="Wrap_NTS99-~11" xfId="153"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1467,7 +1466,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Rail shipments 93-97"/>
@@ -1548,9 +1547,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1588,9 +1587,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1625,7 +1624,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1660,7 +1659,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1833,12 +1832,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B59"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="11.59765625" customWidth="1"/>
-    <col min="2" max="2" width="85.06640625" customWidth="1"/>
+    <col min="1" max="1" width="11.5703125" customWidth="1"/>
+    <col min="2" max="2" width="85" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -2094,8 +2093,8 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B7" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="B14" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="B7" r:id="rId1"/>
+    <hyperlink ref="B14" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId3"/>
@@ -2103,13 +2102,13 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C69"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="73.59765625" customWidth="1"/>
+    <col min="1" max="1" width="73.5703125" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="102.265625" customWidth="1"/>
+    <col min="3" max="3" width="102.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2624,18 +2623,18 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:BE7"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.06640625" customWidth="1"/>
-    <col min="2" max="2" width="8.73046875" customWidth="1"/>
+    <col min="1" max="1" width="13" customWidth="1"/>
+    <col min="2" max="2" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:57" ht="42.75">
+    <row r="1" spans="1:57" ht="45">
       <c r="A1" s="16" t="s">
         <v>111</v>
       </c>
@@ -2813,227 +2812,227 @@
         <v>12</v>
       </c>
       <c r="B2" s="7">
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="C2" s="7">
         <f>$B2</f>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="D2" s="7">
         <f t="shared" ref="D2:AL7" si="0">$B2</f>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="E2" s="7">
         <f t="shared" si="0"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="F2" s="7">
         <f t="shared" si="0"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="G2" s="7">
         <f t="shared" si="0"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="H2" s="7">
         <f t="shared" si="0"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="I2" s="7">
         <f t="shared" si="0"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="J2" s="7">
         <f t="shared" si="0"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="K2" s="7">
         <f t="shared" si="0"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="L2" s="7">
         <f t="shared" si="0"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="M2" s="7">
         <f t="shared" si="0"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="N2" s="7">
         <f t="shared" si="0"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="O2" s="7">
         <f t="shared" si="0"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="P2" s="7">
         <f t="shared" si="0"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="Q2" s="7">
         <f t="shared" si="0"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="R2" s="7">
         <f t="shared" si="0"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="S2" s="7">
         <f t="shared" si="0"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="T2" s="7">
         <f t="shared" si="0"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="U2" s="7">
         <f t="shared" si="0"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="V2" s="7">
         <f t="shared" si="0"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="W2" s="7">
         <f t="shared" si="0"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="X2" s="7">
         <f t="shared" si="0"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="Y2" s="7">
         <f t="shared" si="0"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="Z2" s="7">
         <f t="shared" si="0"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="AA2" s="7">
         <f t="shared" si="0"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="AB2" s="7">
         <f t="shared" si="0"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="AC2" s="7">
         <f t="shared" si="0"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="AD2" s="7">
         <f t="shared" si="0"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="AE2" s="7">
         <f t="shared" si="0"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="AF2" s="7">
         <f t="shared" si="0"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="AG2" s="7">
         <f t="shared" si="0"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="AH2" s="7">
         <f t="shared" si="0"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="AI2" s="7">
         <f t="shared" si="0"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="AJ2" s="7">
         <f t="shared" si="0"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="AK2" s="7">
         <f t="shared" si="0"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="AL2" s="7">
         <f t="shared" si="0"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="AM2" s="7">
         <f t="shared" ref="AL2:BE7" si="1">$B2</f>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="AN2" s="7">
         <f t="shared" si="1"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="AO2" s="7">
         <f t="shared" si="1"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="AP2" s="7">
         <f t="shared" si="1"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="AQ2" s="7">
         <f t="shared" si="1"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="AR2" s="7">
         <f t="shared" si="1"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="AS2" s="7">
         <f t="shared" si="1"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="AT2" s="7">
         <f t="shared" si="1"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="AU2" s="7">
         <f t="shared" si="1"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="AV2" s="7">
         <f t="shared" si="1"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="AW2" s="7">
         <f t="shared" si="1"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="AX2" s="7">
         <f t="shared" si="1"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="AY2" s="7">
         <f t="shared" si="1"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="AZ2" s="7">
         <f t="shared" si="1"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="BA2" s="7">
         <f t="shared" si="1"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="BB2" s="7">
         <f t="shared" si="1"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="BC2" s="7">
         <f t="shared" si="1"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="BD2" s="7">
         <f t="shared" si="1"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="BE2" s="7">
         <f t="shared" si="1"/>
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="3" spans="1:57">
@@ -4186,17 +4185,17 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:BD7"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="11.796875" customWidth="1"/>
+    <col min="1" max="1" width="11.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:56" s="1" customFormat="1" ht="42.75">
+    <row r="1" spans="1:56" s="1" customFormat="1" ht="45">
       <c r="A1" s="16" t="s">
         <v>112</v>
       </c>

</xml_diff>